<commit_message>
continue panchapale and ukhu kheti valuation
</commit_message>
<xml_diff>
--- a/बजेट माग estimate/वडा बजेट estimate/ukhu kheti/valuation ukhu kheti.xlsx
+++ b/बजेट माग estimate/वडा बजेट estimate/ukhu kheti/valuation ukhu kheti.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1920F364-AF7B-4996-8116-9CE5BE177768}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B624F5A-D265-47C2-95AE-ABBF63B02D8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,7 +44,7 @@
     <definedName name="description_783">[1]Abstract!$B$301</definedName>
     <definedName name="description_784">[3]Abstract!$B$300</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">estimate!$A$1:$K$70</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">V!$A$1:$K$70</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">V!$A$1:$K$79</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">estimate!$1:$8</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">V!$1:$8</definedName>
   </definedNames>
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="74">
   <si>
     <t>Government of Nepal</t>
   </si>
@@ -270,6 +270,33 @@
   </si>
   <si>
     <t>Total Valuated</t>
+  </si>
+  <si>
+    <t>-MS square pipe of 3" * 3" of 1.6mm thickness for vertical post</t>
+  </si>
+  <si>
+    <t>-MS square pipe of 66mm*33mm of 1.4mm thickness for vertical post</t>
+  </si>
+  <si>
+    <t>-MS square pipe of 2" * 2" of 1.4mm thickness for vertical post</t>
+  </si>
+  <si>
+    <t>-MS square pipe of 2" * 2" of 1.4mm thickness for purlins</t>
+  </si>
+  <si>
+    <t>-MS square pipe of 3" * 3" of 1.6mm thickness for vertical post for cooking area</t>
+  </si>
+  <si>
+    <t>-MS square pipe of 1.5" * 1.5" of 1.2mm thickness for purlins</t>
+  </si>
+  <si>
+    <t>-MS square pipe of 1.5" * 1.5" of 1.2mm thickness for horizontal support in mid-height section</t>
+  </si>
+  <si>
+    <t>-MS square pipe of 2" * 2" of 1.4mm thickness for horizontal support of roof</t>
+  </si>
+  <si>
+    <t>-cooking area</t>
   </si>
 </sst>
 </file>
@@ -362,7 +389,7 @@
       <name val="Preeti"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -372,6 +399,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -443,7 +476,7 @@
     <xf numFmtId="9" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -556,24 +589,6 @@
     <xf numFmtId="0" fontId="12" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -592,6 +607,45 @@
     </xf>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="4" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="3" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -1138,113 +1192,113 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A1" s="46" t="s">
+      <c r="A1" s="51" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-      <c r="F1" s="46"/>
-      <c r="G1" s="46"/>
-      <c r="H1" s="46"/>
-      <c r="I1" s="46"/>
-      <c r="J1" s="46"/>
-      <c r="K1" s="46"/>
+      <c r="B1" s="51"/>
+      <c r="C1" s="51"/>
+      <c r="D1" s="51"/>
+      <c r="E1" s="51"/>
+      <c r="F1" s="51"/>
+      <c r="G1" s="51"/>
+      <c r="H1" s="51"/>
+      <c r="I1" s="51"/>
+      <c r="J1" s="51"/>
+      <c r="K1" s="51"/>
     </row>
     <row r="2" spans="1:18" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="47" t="s">
+      <c r="A2" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="47"/>
-      <c r="C2" s="47"/>
-      <c r="D2" s="47"/>
-      <c r="E2" s="47"/>
-      <c r="F2" s="47"/>
-      <c r="G2" s="47"/>
-      <c r="H2" s="47"/>
-      <c r="I2" s="47"/>
-      <c r="J2" s="47"/>
-      <c r="K2" s="47"/>
+      <c r="B2" s="52"/>
+      <c r="C2" s="52"/>
+      <c r="D2" s="52"/>
+      <c r="E2" s="52"/>
+      <c r="F2" s="52"/>
+      <c r="G2" s="52"/>
+      <c r="H2" s="52"/>
+      <c r="I2" s="52"/>
+      <c r="J2" s="52"/>
+      <c r="K2" s="52"/>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A3" s="48" t="s">
+      <c r="A3" s="53" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="48"/>
-      <c r="C3" s="48"/>
-      <c r="D3" s="48"/>
-      <c r="E3" s="48"/>
-      <c r="F3" s="48"/>
-      <c r="G3" s="48"/>
-      <c r="H3" s="48"/>
-      <c r="I3" s="48"/>
-      <c r="J3" s="48"/>
-      <c r="K3" s="48"/>
+      <c r="B3" s="53"/>
+      <c r="C3" s="53"/>
+      <c r="D3" s="53"/>
+      <c r="E3" s="53"/>
+      <c r="F3" s="53"/>
+      <c r="G3" s="53"/>
+      <c r="H3" s="53"/>
+      <c r="I3" s="53"/>
+      <c r="J3" s="53"/>
+      <c r="K3" s="53"/>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A4" s="48" t="s">
+      <c r="A4" s="53" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="48"/>
-      <c r="C4" s="48"/>
-      <c r="D4" s="48"/>
-      <c r="E4" s="48"/>
-      <c r="F4" s="48"/>
-      <c r="G4" s="48"/>
-      <c r="H4" s="48"/>
-      <c r="I4" s="48"/>
-      <c r="J4" s="48"/>
-      <c r="K4" s="48"/>
+      <c r="B4" s="53"/>
+      <c r="C4" s="53"/>
+      <c r="D4" s="53"/>
+      <c r="E4" s="53"/>
+      <c r="F4" s="53"/>
+      <c r="G4" s="53"/>
+      <c r="H4" s="53"/>
+      <c r="I4" s="53"/>
+      <c r="J4" s="53"/>
+      <c r="K4" s="53"/>
     </row>
     <row r="5" spans="1:18" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A5" s="49" t="s">
+      <c r="A5" s="54" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="49"/>
-      <c r="C5" s="49"/>
-      <c r="D5" s="49"/>
-      <c r="E5" s="49"/>
-      <c r="F5" s="49"/>
-      <c r="G5" s="49"/>
-      <c r="H5" s="49"/>
-      <c r="I5" s="49"/>
-      <c r="J5" s="49"/>
-      <c r="K5" s="49"/>
+      <c r="B5" s="54"/>
+      <c r="C5" s="54"/>
+      <c r="D5" s="54"/>
+      <c r="E5" s="54"/>
+      <c r="F5" s="54"/>
+      <c r="G5" s="54"/>
+      <c r="H5" s="54"/>
+      <c r="I5" s="54"/>
+      <c r="J5" s="54"/>
+      <c r="K5" s="54"/>
     </row>
     <row r="6" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="44" t="s">
+      <c r="A6" s="55" t="s">
         <v>60</v>
       </c>
-      <c r="B6" s="44"/>
-      <c r="C6" s="44"/>
-      <c r="D6" s="44"/>
-      <c r="E6" s="44"/>
-      <c r="F6" s="44"/>
+      <c r="B6" s="55"/>
+      <c r="C6" s="55"/>
+      <c r="D6" s="55"/>
+      <c r="E6" s="55"/>
+      <c r="F6" s="55"/>
       <c r="G6" s="10"/>
-      <c r="H6" s="45" t="s">
+      <c r="H6" s="56" t="s">
         <v>25</v>
       </c>
-      <c r="I6" s="45"/>
-      <c r="J6" s="45"/>
-      <c r="K6" s="45"/>
+      <c r="I6" s="56"/>
+      <c r="J6" s="56"/>
+      <c r="K6" s="56"/>
     </row>
     <row r="7" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="52" t="s">
+      <c r="A7" s="46" t="s">
         <v>48</v>
       </c>
-      <c r="B7" s="52"/>
-      <c r="C7" s="52"/>
-      <c r="D7" s="52"/>
-      <c r="E7" s="52"/>
-      <c r="F7" s="52"/>
+      <c r="B7" s="46"/>
+      <c r="C7" s="46"/>
+      <c r="D7" s="46"/>
+      <c r="E7" s="46"/>
+      <c r="F7" s="46"/>
       <c r="G7" s="11"/>
-      <c r="H7" s="53" t="s">
+      <c r="H7" s="47" t="s">
         <v>61</v>
       </c>
-      <c r="I7" s="53"/>
-      <c r="J7" s="53"/>
-      <c r="K7" s="53"/>
+      <c r="I7" s="47"/>
+      <c r="J7" s="47"/>
+      <c r="K7" s="47"/>
     </row>
     <row r="8" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
@@ -2513,11 +2567,11 @@
       <c r="B65" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="C65" s="50">
+      <c r="C65" s="44">
         <f>J63</f>
         <v>234835.07491669987</v>
       </c>
-      <c r="D65" s="51"/>
+      <c r="D65" s="45"/>
       <c r="E65" s="9">
         <v>100</v>
       </c>
@@ -2539,21 +2593,21 @@
       <c r="B66" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="C66" s="54">
+      <c r="C66" s="48">
         <v>200000</v>
       </c>
-      <c r="D66" s="55"/>
+      <c r="D66" s="49"/>
       <c r="E66" s="9"/>
     </row>
     <row r="67" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B67" s="27" t="s">
         <v>22</v>
       </c>
-      <c r="C67" s="54">
+      <c r="C67" s="48">
         <f>C66-C69-C70</f>
         <v>190000</v>
       </c>
-      <c r="D67" s="55"/>
+      <c r="D67" s="49"/>
       <c r="E67" s="9">
         <f>C67/C65*100</f>
         <v>80.907845673137345</v>
@@ -2563,11 +2617,11 @@
       <c r="B68" s="27" t="s">
         <v>31</v>
       </c>
-      <c r="C68" s="56">
+      <c r="C68" s="50">
         <f>C65-C67</f>
         <v>44835.074916699872</v>
       </c>
-      <c r="D68" s="56"/>
+      <c r="D68" s="50"/>
       <c r="E68" s="9">
         <f>100-E67</f>
         <v>19.092154326862655</v>
@@ -2577,11 +2631,11 @@
       <c r="B69" s="27" t="s">
         <v>23</v>
       </c>
-      <c r="C69" s="50">
+      <c r="C69" s="44">
         <f>C66*0.03</f>
         <v>6000</v>
       </c>
-      <c r="D69" s="51"/>
+      <c r="D69" s="45"/>
       <c r="E69" s="9">
         <v>3</v>
       </c>
@@ -2590,17 +2644,24 @@
       <c r="B70" s="27" t="s">
         <v>24</v>
       </c>
-      <c r="C70" s="50">
+      <c r="C70" s="44">
         <f>C66*0.02</f>
         <v>4000</v>
       </c>
-      <c r="D70" s="51"/>
+      <c r="D70" s="45"/>
       <c r="E70" s="9">
         <v>2</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="H6:K6"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A4:K4"/>
+    <mergeCell ref="A5:K5"/>
     <mergeCell ref="C69:D69"/>
     <mergeCell ref="C70:D70"/>
     <mergeCell ref="A7:F7"/>
@@ -2609,13 +2670,6 @@
     <mergeCell ref="C66:D66"/>
     <mergeCell ref="C67:D67"/>
     <mergeCell ref="C68:D68"/>
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="H6:K6"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A3:K3"/>
-    <mergeCell ref="A4:K4"/>
-    <mergeCell ref="A5:K5"/>
   </mergeCells>
   <pageMargins left="0.70866141732283505" right="0.70866141732283505" top="0.74803149606299202" bottom="0.74803149606299202" header="0.31496062992126" footer="0.31496062992126"/>
   <pageSetup paperSize="9" scale="80" orientation="portrait" verticalDpi="1200" r:id="rId1"/>
@@ -2630,7 +2684,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD9D6B52-0BCE-4A59-BC99-2ABBFC24DADE}">
-  <dimension ref="A1:S70"/>
+  <dimension ref="A1:S79"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4.7109375" style="19" customWidth="1"/>
@@ -2648,116 +2702,116 @@
     <col min="17" max="16384" width="9.140625" style="19"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A1" s="46" t="s">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" s="51" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-      <c r="F1" s="46"/>
-      <c r="G1" s="46"/>
-      <c r="H1" s="46"/>
-      <c r="I1" s="46"/>
-      <c r="J1" s="46"/>
-      <c r="K1" s="46"/>
-    </row>
-    <row r="2" spans="1:18" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="47" t="s">
+      <c r="B1" s="51"/>
+      <c r="C1" s="51"/>
+      <c r="D1" s="51"/>
+      <c r="E1" s="51"/>
+      <c r="F1" s="51"/>
+      <c r="G1" s="51"/>
+      <c r="H1" s="51"/>
+      <c r="I1" s="51"/>
+      <c r="J1" s="51"/>
+      <c r="K1" s="51"/>
+    </row>
+    <row r="2" spans="1:11" ht="22.5" x14ac:dyDescent="0.25">
+      <c r="A2" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="47"/>
-      <c r="C2" s="47"/>
-      <c r="D2" s="47"/>
-      <c r="E2" s="47"/>
-      <c r="F2" s="47"/>
-      <c r="G2" s="47"/>
-      <c r="H2" s="47"/>
-      <c r="I2" s="47"/>
-      <c r="J2" s="47"/>
-      <c r="K2" s="47"/>
-    </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A3" s="48" t="s">
+      <c r="B2" s="52"/>
+      <c r="C2" s="52"/>
+      <c r="D2" s="52"/>
+      <c r="E2" s="52"/>
+      <c r="F2" s="52"/>
+      <c r="G2" s="52"/>
+      <c r="H2" s="52"/>
+      <c r="I2" s="52"/>
+      <c r="J2" s="52"/>
+      <c r="K2" s="52"/>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" s="53" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="48"/>
-      <c r="C3" s="48"/>
-      <c r="D3" s="48"/>
-      <c r="E3" s="48"/>
-      <c r="F3" s="48"/>
-      <c r="G3" s="48"/>
-      <c r="H3" s="48"/>
-      <c r="I3" s="48"/>
-      <c r="J3" s="48"/>
-      <c r="K3" s="48"/>
-    </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A4" s="48" t="s">
+      <c r="B3" s="53"/>
+      <c r="C3" s="53"/>
+      <c r="D3" s="53"/>
+      <c r="E3" s="53"/>
+      <c r="F3" s="53"/>
+      <c r="G3" s="53"/>
+      <c r="H3" s="53"/>
+      <c r="I3" s="53"/>
+      <c r="J3" s="53"/>
+      <c r="K3" s="53"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" s="53" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="48"/>
-      <c r="C4" s="48"/>
-      <c r="D4" s="48"/>
-      <c r="E4" s="48"/>
-      <c r="F4" s="48"/>
-      <c r="G4" s="48"/>
-      <c r="H4" s="48"/>
-      <c r="I4" s="48"/>
-      <c r="J4" s="48"/>
-      <c r="K4" s="48"/>
-    </row>
-    <row r="5" spans="1:18" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A5" s="49" t="s">
+      <c r="B4" s="53"/>
+      <c r="C4" s="53"/>
+      <c r="D4" s="53"/>
+      <c r="E4" s="53"/>
+      <c r="F4" s="53"/>
+      <c r="G4" s="53"/>
+      <c r="H4" s="53"/>
+      <c r="I4" s="53"/>
+      <c r="J4" s="53"/>
+      <c r="K4" s="53"/>
+    </row>
+    <row r="5" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A5" s="54" t="s">
         <v>63</v>
       </c>
-      <c r="B5" s="49"/>
-      <c r="C5" s="49"/>
-      <c r="D5" s="49"/>
-      <c r="E5" s="49"/>
-      <c r="F5" s="49"/>
-      <c r="G5" s="49"/>
-      <c r="H5" s="49"/>
-      <c r="I5" s="49"/>
-      <c r="J5" s="49"/>
-      <c r="K5" s="49"/>
-    </row>
-    <row r="6" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="44" t="s">
+      <c r="B5" s="54"/>
+      <c r="C5" s="54"/>
+      <c r="D5" s="54"/>
+      <c r="E5" s="54"/>
+      <c r="F5" s="54"/>
+      <c r="G5" s="54"/>
+      <c r="H5" s="54"/>
+      <c r="I5" s="54"/>
+      <c r="J5" s="54"/>
+      <c r="K5" s="54"/>
+    </row>
+    <row r="6" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A6" s="55" t="s">
         <v>60</v>
       </c>
-      <c r="B6" s="44"/>
-      <c r="C6" s="44"/>
-      <c r="D6" s="44"/>
-      <c r="E6" s="44"/>
-      <c r="F6" s="44"/>
+      <c r="B6" s="55"/>
+      <c r="C6" s="55"/>
+      <c r="D6" s="55"/>
+      <c r="E6" s="55"/>
+      <c r="F6" s="55"/>
       <c r="G6" s="10"/>
-      <c r="H6" s="45" t="s">
+      <c r="H6" s="56" t="s">
         <v>25</v>
       </c>
-      <c r="I6" s="45"/>
-      <c r="J6" s="45"/>
-      <c r="K6" s="45"/>
-    </row>
-    <row r="7" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="52" t="s">
+      <c r="I6" s="56"/>
+      <c r="J6" s="56"/>
+      <c r="K6" s="56"/>
+    </row>
+    <row r="7" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A7" s="46" t="s">
         <v>48</v>
       </c>
-      <c r="B7" s="52"/>
-      <c r="C7" s="52"/>
-      <c r="D7" s="52"/>
-      <c r="E7" s="52"/>
-      <c r="F7" s="52"/>
+      <c r="B7" s="46"/>
+      <c r="C7" s="46"/>
+      <c r="D7" s="46"/>
+      <c r="E7" s="46"/>
+      <c r="F7" s="46"/>
       <c r="G7" s="11"/>
-      <c r="H7" s="53" t="s">
+      <c r="H7" s="47" t="s">
         <v>61</v>
       </c>
-      <c r="I7" s="53"/>
-      <c r="J7" s="53"/>
-      <c r="K7" s="53"/>
-    </row>
-    <row r="8" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="I7" s="47"/>
+      <c r="J7" s="47"/>
+      <c r="K7" s="47"/>
+    </row>
+    <row r="8" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
         <v>5</v>
       </c>
@@ -2792,7 +2846,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:18" s="35" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" s="35" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>1</v>
       </c>
@@ -2817,433 +2871,457 @@
       <c r="J9" s="39"/>
       <c r="K9" s="5"/>
     </row>
-    <row r="10" spans="1:18" s="35" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" s="35" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="16"/>
       <c r="B10" s="40" t="s">
-        <v>57</v>
-      </c>
-      <c r="C10" s="41">
-        <f>2*3</f>
-        <v>6</v>
-      </c>
-      <c r="D10" s="9">
-        <f>(11+1+2)/3.281</f>
-        <v>4.2669917708015843</v>
-      </c>
-      <c r="E10" s="9">
-        <v>4.4000000000000004</v>
-      </c>
-      <c r="F10" s="9">
-        <f t="shared" ref="F10:F16" si="0">PRODUCT(C10:E10)</f>
-        <v>112.64858274916183</v>
-      </c>
-      <c r="G10" s="9">
-        <f t="shared" ref="G10:G16" si="1">F10</f>
-        <v>112.64858274916183</v>
+        <v>65</v>
+      </c>
+      <c r="C10" s="63">
+        <v>2</v>
+      </c>
+      <c r="D10" s="64">
+        <f>(15.5+1)/3.281</f>
+        <v>5.0289545870161536</v>
+      </c>
+      <c r="E10" s="64">
+        <v>3.54</v>
+      </c>
+      <c r="F10" s="64">
+        <f t="shared" ref="F10" si="0">PRODUCT(C10:E10)</f>
+        <v>35.604998476074371</v>
+      </c>
+      <c r="G10" s="64">
+        <f t="shared" ref="G10" si="1">F10</f>
+        <v>35.604998476074371</v>
       </c>
       <c r="H10" s="39"/>
       <c r="I10" s="39"/>
       <c r="J10" s="39"/>
       <c r="K10" s="27"/>
     </row>
-    <row r="11" spans="1:18" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" s="35" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="16"/>
       <c r="B11" s="40"/>
-      <c r="C11" s="41">
-        <f>2*3</f>
-        <v>6</v>
-      </c>
-      <c r="D11" s="9">
-        <f>(11+1+1+2)/3.281</f>
-        <v>4.5717768972874122</v>
-      </c>
-      <c r="E11" s="9">
-        <v>4.4000000000000004</v>
-      </c>
-      <c r="F11" s="9">
-        <f t="shared" si="0"/>
-        <v>120.69491008838769</v>
-      </c>
-      <c r="G11" s="9">
-        <f t="shared" si="1"/>
-        <v>120.69491008838769</v>
+      <c r="C11" s="63">
+        <v>2</v>
+      </c>
+      <c r="D11" s="64">
+        <f>(15.5-1.5+2)/3.281</f>
+        <v>4.8765620237732392</v>
+      </c>
+      <c r="E11" s="64">
+        <v>3.54</v>
+      </c>
+      <c r="F11" s="64">
+        <f t="shared" ref="F11" si="2">PRODUCT(C11:E11)</f>
+        <v>34.526059128314536</v>
+      </c>
+      <c r="G11" s="64">
+        <f t="shared" ref="G11" si="3">F11</f>
+        <v>34.526059128314536</v>
       </c>
       <c r="H11" s="39"/>
       <c r="I11" s="39"/>
       <c r="J11" s="39"/>
       <c r="K11" s="27"/>
     </row>
-    <row r="12" spans="1:18" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" s="35" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="16"/>
-      <c r="B12" s="40"/>
-      <c r="C12" s="41">
-        <f>2</f>
+      <c r="B12" s="40" t="s">
+        <v>67</v>
+      </c>
+      <c r="C12" s="63">
         <v>2</v>
       </c>
-      <c r="D12" s="9">
-        <f>(11+1+2)/3.281</f>
-        <v>4.2669917708015843</v>
-      </c>
-      <c r="E12" s="9">
-        <v>4.4000000000000004</v>
-      </c>
-      <c r="F12" s="9">
-        <f t="shared" si="0"/>
-        <v>37.549527583053944</v>
-      </c>
-      <c r="G12" s="9">
-        <f t="shared" si="1"/>
-        <v>37.549527583053944</v>
+      <c r="D12" s="64">
+        <v>3.9</v>
+      </c>
+      <c r="E12" s="64">
+        <v>2.14</v>
+      </c>
+      <c r="F12" s="64">
+        <f>PRODUCT(C12:E12)</f>
+        <v>16.692</v>
+      </c>
+      <c r="G12" s="64">
+        <f>F12</f>
+        <v>16.692</v>
       </c>
       <c r="H12" s="39"/>
       <c r="I12" s="39"/>
       <c r="J12" s="39"/>
       <c r="K12" s="27"/>
     </row>
-    <row r="13" spans="1:18" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" s="35" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="16"/>
-      <c r="B13" s="40"/>
-      <c r="C13" s="41">
-        <f>2</f>
-        <v>2</v>
-      </c>
-      <c r="D13" s="9">
-        <f>(11+1+1+2)/3.281</f>
-        <v>4.5717768972874122</v>
-      </c>
-      <c r="E13" s="9">
-        <v>4.4000000000000004</v>
-      </c>
-      <c r="F13" s="9">
-        <f t="shared" si="0"/>
-        <v>40.231636696129229</v>
-      </c>
-      <c r="G13" s="9">
-        <f t="shared" si="1"/>
-        <v>40.231636696129229</v>
+      <c r="B13" s="40" t="s">
+        <v>68</v>
+      </c>
+      <c r="C13" s="63">
+        <v>9</v>
+      </c>
+      <c r="D13" s="64">
+        <v>3.09</v>
+      </c>
+      <c r="E13" s="64">
+        <v>2.14</v>
+      </c>
+      <c r="F13" s="64">
+        <f t="shared" ref="F13" si="4">PRODUCT(C13:E13)</f>
+        <v>59.513399999999997</v>
+      </c>
+      <c r="G13" s="64">
+        <f t="shared" ref="G13" si="5">F13</f>
+        <v>59.513399999999997</v>
       </c>
       <c r="H13" s="39"/>
       <c r="I13" s="39"/>
       <c r="J13" s="39"/>
       <c r="K13" s="27"/>
     </row>
-    <row r="14" spans="1:18" s="35" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" s="35" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A14" s="16"/>
       <c r="B14" s="40" t="s">
-        <v>58</v>
-      </c>
-      <c r="C14" s="41">
-        <f>2*(2+1)</f>
-        <v>6</v>
-      </c>
-      <c r="D14" s="9">
-        <f>(12+3)/3.281</f>
-        <v>4.5717768972874122</v>
-      </c>
-      <c r="E14" s="9">
-        <v>3.01</v>
-      </c>
-      <c r="F14" s="9">
-        <f t="shared" si="0"/>
-        <v>82.566290765010663</v>
-      </c>
-      <c r="G14" s="9">
-        <f t="shared" si="1"/>
-        <v>82.566290765010663</v>
+        <v>66</v>
+      </c>
+      <c r="C14" s="63">
+        <v>1</v>
+      </c>
+      <c r="D14" s="64">
+        <v>3.9</v>
+      </c>
+      <c r="E14" s="64">
+        <v>2.35</v>
+      </c>
+      <c r="F14" s="64">
+        <f t="shared" ref="F14" si="6">PRODUCT(C14:E14)</f>
+        <v>9.1650000000000009</v>
+      </c>
+      <c r="G14" s="64">
+        <f t="shared" ref="G14" si="7">F14</f>
+        <v>9.1650000000000009</v>
       </c>
       <c r="H14" s="39"/>
       <c r="I14" s="39"/>
       <c r="J14" s="39"/>
       <c r="K14" s="27"/>
-      <c r="Q14" s="35">
-        <f>PRODUCT(C14:D14)</f>
-        <v>27.430661383724473</v>
-      </c>
-      <c r="R14" s="35">
-        <f>CONVERT(Q14,"m","ft")</f>
-        <v>89.995608214319134</v>
-      </c>
-    </row>
-    <row r="15" spans="1:18" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="15" spans="1:11" s="35" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A15" s="16"/>
-      <c r="B15" s="40"/>
-      <c r="C15" s="41">
-        <f>2*(2+1)</f>
-        <v>6</v>
-      </c>
-      <c r="D15" s="9">
-        <f>(10+3)/3.281</f>
-        <v>3.9622066443157573</v>
-      </c>
-      <c r="E15" s="9">
-        <v>3.01</v>
-      </c>
-      <c r="F15" s="9">
-        <f t="shared" si="0"/>
-        <v>71.557451996342579</v>
-      </c>
-      <c r="G15" s="9">
-        <f t="shared" si="1"/>
-        <v>71.557451996342579</v>
+      <c r="B15" s="40" t="s">
+        <v>69</v>
+      </c>
+      <c r="C15" s="63">
+        <v>3</v>
+      </c>
+      <c r="D15" s="64">
+        <f>(7+1)/3.281</f>
+        <v>2.4382810118866196</v>
+      </c>
+      <c r="E15" s="64">
+        <v>3.54</v>
+      </c>
+      <c r="F15" s="64">
+        <f t="shared" ref="F15" si="8">PRODUCT(C15:E15)</f>
+        <v>25.8945443462359</v>
+      </c>
+      <c r="G15" s="64">
+        <f t="shared" ref="G15" si="9">F15</f>
+        <v>25.8945443462359</v>
       </c>
       <c r="H15" s="39"/>
       <c r="I15" s="39"/>
       <c r="J15" s="39"/>
       <c r="K15" s="27"/>
     </row>
-    <row r="16" spans="1:18" s="35" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" s="35" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="16"/>
-      <c r="B16" s="40" t="s">
-        <v>59</v>
-      </c>
-      <c r="C16" s="41">
-        <f>2*2</f>
-        <v>4</v>
-      </c>
-      <c r="D16" s="9">
-        <f>(12+3)/3.281</f>
-        <v>4.5717768972874122</v>
-      </c>
-      <c r="E16" s="9">
-        <v>2.2599999999999998</v>
-      </c>
-      <c r="F16" s="9">
-        <f t="shared" si="0"/>
-        <v>41.328863151478203</v>
-      </c>
-      <c r="G16" s="9">
-        <f t="shared" si="1"/>
-        <v>41.328863151478203</v>
+      <c r="B16" s="40"/>
+      <c r="C16" s="63">
+        <v>3</v>
+      </c>
+      <c r="D16" s="64">
+        <v>2.6</v>
+      </c>
+      <c r="E16" s="64">
+        <v>3.54</v>
+      </c>
+      <c r="F16" s="64">
+        <f t="shared" ref="F16:F17" si="10">PRODUCT(C16:E16)</f>
+        <v>27.612000000000002</v>
+      </c>
+      <c r="G16" s="64">
+        <f t="shared" ref="G16:G17" si="11">F16</f>
+        <v>27.612000000000002</v>
       </c>
       <c r="H16" s="39"/>
       <c r="I16" s="39"/>
       <c r="J16" s="39"/>
       <c r="K16" s="27"/>
     </row>
-    <row r="17" spans="1:11" s="35" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="2"/>
+    <row r="17" spans="1:11" s="35" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A17" s="16"/>
       <c r="B17" s="40" t="s">
+        <v>70</v>
+      </c>
+      <c r="C17" s="63">
+        <v>5</v>
+      </c>
+      <c r="D17" s="64">
+        <v>3.09</v>
+      </c>
+      <c r="E17" s="64">
+        <v>1.39</v>
+      </c>
+      <c r="F17" s="64">
+        <f t="shared" si="10"/>
+        <v>21.475499999999997</v>
+      </c>
+      <c r="G17" s="64">
+        <f t="shared" si="11"/>
+        <v>21.475499999999997</v>
+      </c>
+      <c r="H17" s="39"/>
+      <c r="I17" s="39"/>
+      <c r="J17" s="39"/>
+      <c r="K17" s="27"/>
+    </row>
+    <row r="18" spans="1:11" s="35" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="A18" s="16"/>
+      <c r="B18" s="40" t="s">
+        <v>71</v>
+      </c>
+      <c r="C18" s="63">
+        <v>5</v>
+      </c>
+      <c r="D18" s="64">
+        <f>1.8+1.9</f>
+        <v>3.7</v>
+      </c>
+      <c r="E18" s="64">
+        <v>1.39</v>
+      </c>
+      <c r="F18" s="64">
+        <f t="shared" ref="F18" si="12">PRODUCT(C18:E18)</f>
+        <v>25.715</v>
+      </c>
+      <c r="G18" s="64">
+        <f t="shared" ref="G18" si="13">F18</f>
+        <v>25.715</v>
+      </c>
+      <c r="H18" s="39"/>
+      <c r="I18" s="39"/>
+      <c r="J18" s="39"/>
+      <c r="K18" s="27"/>
+    </row>
+    <row r="19" spans="1:11" s="35" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="A19" s="16"/>
+      <c r="B19" s="40" t="s">
+        <v>72</v>
+      </c>
+      <c r="C19" s="63">
+        <v>3</v>
+      </c>
+      <c r="D19" s="64">
+        <f>13/3.281</f>
+        <v>3.9622066443157573</v>
+      </c>
+      <c r="E19" s="64">
+        <v>1.39</v>
+      </c>
+      <c r="F19" s="64">
+        <f t="shared" ref="F19" si="14">PRODUCT(C19:E19)</f>
+        <v>16.522401706796707</v>
+      </c>
+      <c r="G19" s="64">
+        <f t="shared" ref="G19" si="15">F19</f>
+        <v>16.522401706796707</v>
+      </c>
+      <c r="H19" s="39"/>
+      <c r="I19" s="39"/>
+      <c r="J19" s="39"/>
+      <c r="K19" s="27"/>
+    </row>
+    <row r="20" spans="1:11" s="35" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="2"/>
+      <c r="B20" s="40" t="s">
         <v>36</v>
-      </c>
-      <c r="C17" s="3"/>
-      <c r="D17" s="4"/>
-      <c r="E17" s="5"/>
-      <c r="F17" s="5"/>
-      <c r="G17" s="39">
-        <f>SUM(G10:G16)</f>
-        <v>506.57726302956416</v>
-      </c>
-      <c r="H17" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="I17" s="6">
-        <v>182.51</v>
-      </c>
-      <c r="J17" s="39">
-        <f>G17*I17</f>
-        <v>92455.416275525757</v>
-      </c>
-      <c r="K17" s="5"/>
-    </row>
-    <row r="18" spans="1:11" s="35" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="2"/>
-      <c r="B18" s="40" t="s">
-        <v>38</v>
-      </c>
-      <c r="C18" s="3"/>
-      <c r="D18" s="4"/>
-      <c r="E18" s="5"/>
-      <c r="F18" s="5"/>
-      <c r="G18" s="39"/>
-      <c r="H18" s="7"/>
-      <c r="I18" s="6"/>
-      <c r="J18" s="39">
-        <f>0.13*G17*(1871.42/18.94)</f>
-        <v>6506.9929675418325</v>
-      </c>
-      <c r="K18" s="5"/>
-    </row>
-    <row r="19" spans="1:11" s="35" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="2"/>
-      <c r="B19" s="40"/>
-      <c r="C19" s="3"/>
-      <c r="D19" s="4"/>
-      <c r="E19" s="5"/>
-      <c r="F19" s="5"/>
-      <c r="G19" s="39"/>
-      <c r="H19" s="7"/>
-      <c r="I19" s="6"/>
-      <c r="J19" s="39"/>
-      <c r="K19" s="5"/>
-    </row>
-    <row r="20" spans="1:11" s="35" customFormat="1" ht="45" x14ac:dyDescent="0.25">
-      <c r="A20" s="2">
-        <v>2</v>
-      </c>
-      <c r="B20" s="36" t="s">
-        <v>62</v>
       </c>
       <c r="C20" s="3"/>
       <c r="D20" s="4"/>
       <c r="E20" s="5"/>
       <c r="F20" s="5"/>
-      <c r="G20" s="39"/>
-      <c r="H20" s="7"/>
-      <c r="I20" s="6"/>
-      <c r="J20" s="39"/>
+      <c r="G20" s="39">
+        <f>SUM(G10:G19)</f>
+        <v>272.72090365742145</v>
+      </c>
+      <c r="H20" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="I20" s="6">
+        <v>182.51</v>
+      </c>
+      <c r="J20" s="39">
+        <f>G20*I20</f>
+        <v>49774.292126515982</v>
+      </c>
       <c r="K20" s="5"/>
     </row>
     <row r="21" spans="1:11" s="35" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2"/>
       <c r="B21" s="40" t="s">
-        <v>39</v>
-      </c>
-      <c r="C21" s="3">
-        <f>2*1</f>
-        <v>2</v>
-      </c>
-      <c r="D21" s="4">
-        <f>(10+3)/3.281</f>
-        <v>3.9622066443157573</v>
-      </c>
-      <c r="E21" s="5">
-        <f>(12+3)/3.281</f>
-        <v>4.5717768972874122</v>
-      </c>
+        <v>38</v>
+      </c>
+      <c r="C21" s="3"/>
+      <c r="D21" s="4"/>
+      <c r="E21" s="5"/>
       <c r="F21" s="5"/>
-      <c r="G21" s="33">
-        <f t="shared" ref="G21:G22" si="2">PRODUCT(C21:F21)</f>
-        <v>36.228649597522924</v>
-      </c>
+      <c r="G21" s="39"/>
       <c r="H21" s="7"/>
       <c r="I21" s="6"/>
-      <c r="J21" s="39"/>
+      <c r="J21" s="39">
+        <f>0.13*G20*(1871.42/18.94)</f>
+        <v>3503.1043272404604</v>
+      </c>
       <c r="K21" s="5"/>
     </row>
     <row r="22" spans="1:11" s="35" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2"/>
       <c r="B22" s="40"/>
-      <c r="C22" s="3">
-        <v>1</v>
-      </c>
-      <c r="D22" s="4">
-        <f>(10+3)/3.281</f>
-        <v>3.9622066443157573</v>
-      </c>
-      <c r="E22" s="5">
-        <f>(10+3)/3.281</f>
-        <v>3.9622066443157573</v>
-      </c>
+      <c r="C22" s="3"/>
+      <c r="D22" s="4"/>
+      <c r="E22" s="5"/>
       <c r="F22" s="5"/>
-      <c r="G22" s="33">
-        <f t="shared" si="2"/>
-        <v>15.699081492259934</v>
-      </c>
+      <c r="G22" s="39"/>
       <c r="H22" s="7"/>
       <c r="I22" s="6"/>
       <c r="J22" s="39"/>
       <c r="K22" s="5"/>
     </row>
-    <row r="23" spans="1:11" s="35" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="2"/>
-      <c r="B23" s="40" t="s">
-        <v>36</v>
+    <row r="23" spans="1:11" s="35" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="A23" s="2">
+        <v>2</v>
+      </c>
+      <c r="B23" s="36" t="s">
+        <v>62</v>
       </c>
       <c r="C23" s="3"/>
       <c r="D23" s="4"/>
       <c r="E23" s="5"/>
       <c r="F23" s="5"/>
-      <c r="G23" s="39">
-        <f>SUM(G21:G22)</f>
-        <v>51.92773108978286</v>
-      </c>
-      <c r="H23" s="7" t="s">
+      <c r="G23" s="39"/>
+      <c r="H23" s="7"/>
+      <c r="I23" s="6"/>
+      <c r="J23" s="39"/>
+      <c r="K23" s="5"/>
+    </row>
+    <row r="24" spans="1:11" s="35" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="2"/>
+      <c r="B24" s="40" t="s">
+        <v>39</v>
+      </c>
+      <c r="C24" s="60">
+        <f>2*1</f>
+        <v>2</v>
+      </c>
+      <c r="D24" s="61">
+        <f>(10+4)/3.281</f>
+        <v>4.2669917708015843</v>
+      </c>
+      <c r="E24" s="62">
+        <f>(7)/3.281</f>
+        <v>2.1334958854007922</v>
+      </c>
+      <c r="F24" s="62"/>
+      <c r="G24" s="58">
+        <f t="shared" ref="G24:G25" si="16">PRODUCT(C24:F24)</f>
+        <v>18.207218772088439</v>
+      </c>
+      <c r="H24" s="7"/>
+      <c r="I24" s="6"/>
+      <c r="J24" s="39"/>
+      <c r="K24" s="5"/>
+    </row>
+    <row r="25" spans="1:11" s="35" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="2"/>
+      <c r="B25" s="40" t="s">
+        <v>73</v>
+      </c>
+      <c r="C25" s="60">
+        <v>1</v>
+      </c>
+      <c r="D25" s="61">
+        <f>(13.5)/3.281</f>
+        <v>4.1145992075586708</v>
+      </c>
+      <c r="E25" s="62">
+        <f>1.8+1.9</f>
+        <v>3.7</v>
+      </c>
+      <c r="F25" s="62"/>
+      <c r="G25" s="58">
+        <f t="shared" si="16"/>
+        <v>15.224017067967083</v>
+      </c>
+      <c r="H25" s="7"/>
+      <c r="I25" s="6"/>
+      <c r="J25" s="39"/>
+      <c r="K25" s="5"/>
+    </row>
+    <row r="26" spans="1:11" s="35" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="2"/>
+      <c r="B26" s="40"/>
+      <c r="C26" s="60">
+        <v>1</v>
+      </c>
+      <c r="D26" s="61">
+        <f>(7)/3.281</f>
+        <v>2.1334958854007922</v>
+      </c>
+      <c r="E26" s="62">
+        <f>1.8+1.9</f>
+        <v>3.7</v>
+      </c>
+      <c r="F26" s="62"/>
+      <c r="G26" s="58">
+        <f t="shared" ref="G26" si="17">PRODUCT(C26:F26)</f>
+        <v>7.893934775982931</v>
+      </c>
+      <c r="H26" s="7"/>
+      <c r="I26" s="6"/>
+      <c r="J26" s="39"/>
+      <c r="K26" s="5"/>
+    </row>
+    <row r="27" spans="1:11" s="35" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="2"/>
+      <c r="B27" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="C27" s="3"/>
+      <c r="D27" s="4"/>
+      <c r="E27" s="5"/>
+      <c r="F27" s="5"/>
+      <c r="G27" s="39">
+        <f>SUM(G24:G26)</f>
+        <v>41.325170616038449</v>
+      </c>
+      <c r="H27" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="I23" s="6">
+      <c r="I27" s="6">
         <v>1074.98</v>
       </c>
-      <c r="J23" s="39">
-        <f>G23*I23</f>
-        <v>55821.27236689478</v>
-      </c>
-      <c r="K23" s="5"/>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A24" s="16"/>
-      <c r="B24" s="32" t="s">
-        <v>41</v>
-      </c>
-      <c r="C24" s="17"/>
-      <c r="D24" s="17"/>
-      <c r="E24" s="17"/>
-      <c r="F24" s="17"/>
-      <c r="G24" s="17"/>
-      <c r="H24" s="17"/>
-      <c r="I24" s="17"/>
-      <c r="J24" s="18">
-        <f>0.13*G23*6674.66/10</f>
-        <v>4505.7993447444915</v>
-      </c>
-      <c r="K24" s="17"/>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A25" s="16"/>
-      <c r="B25" s="32" t="s">
-        <v>42</v>
-      </c>
-      <c r="C25" s="17"/>
-      <c r="D25" s="17"/>
-      <c r="E25" s="17"/>
-      <c r="F25" s="17"/>
-      <c r="G25" s="17"/>
-      <c r="H25" s="17"/>
-      <c r="I25" s="17"/>
-      <c r="J25" s="18">
-        <f>0.13*G23*1023.75/10</f>
-        <v>691.09319114114771</v>
-      </c>
-      <c r="K25" s="17"/>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A26" s="16"/>
-      <c r="B26" s="32" t="s">
-        <v>43</v>
-      </c>
-      <c r="C26" s="17"/>
-      <c r="D26" s="17"/>
-      <c r="E26" s="17"/>
-      <c r="F26" s="17"/>
-      <c r="G26" s="17"/>
-      <c r="H26" s="17"/>
-      <c r="I26" s="17"/>
-      <c r="J26" s="18">
-        <f>0.13*G23*348.21/10</f>
-        <v>235.06281815605274</v>
-      </c>
-      <c r="K26" s="17"/>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A27" s="16"/>
-      <c r="B27" s="32" t="s">
-        <v>44</v>
-      </c>
-      <c r="C27" s="17"/>
-      <c r="D27" s="17"/>
-      <c r="E27" s="17"/>
-      <c r="F27" s="17"/>
-      <c r="G27" s="17"/>
-      <c r="H27" s="17"/>
-      <c r="I27" s="17"/>
-      <c r="J27" s="18">
-        <f>0.13*G23*165/10</f>
-        <v>111.38498318758425</v>
-      </c>
-      <c r="K27" s="17"/>
+      <c r="J27" s="39">
+        <f>G27*I27</f>
+        <v>44423.73190882901</v>
+      </c>
+      <c r="K27" s="5"/>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="16"/>
-      <c r="B28" s="32"/>
+      <c r="B28" s="32" t="s">
+        <v>41</v>
+      </c>
       <c r="C28" s="17"/>
       <c r="D28" s="17"/>
       <c r="E28" s="17"/>
@@ -3251,15 +3329,16 @@
       <c r="G28" s="17"/>
       <c r="H28" s="17"/>
       <c r="I28" s="17"/>
-      <c r="J28" s="18"/>
+      <c r="J28" s="18">
+        <f>0.13*G27*6674.66/10</f>
+        <v>3585.8090229526133</v>
+      </c>
       <c r="K28" s="17"/>
     </row>
-    <row r="29" spans="1:11" ht="30.75" x14ac:dyDescent="0.25">
-      <c r="A29" s="16">
-        <v>3</v>
-      </c>
-      <c r="B29" s="43" t="s">
-        <v>49</v>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A29" s="16"/>
+      <c r="B29" s="32" t="s">
+        <v>42</v>
       </c>
       <c r="C29" s="17"/>
       <c r="D29" s="17"/>
@@ -3268,92 +3347,68 @@
       <c r="G29" s="17"/>
       <c r="H29" s="17"/>
       <c r="I29" s="17"/>
-      <c r="J29" s="18"/>
+      <c r="J29" s="18">
+        <f>0.13*G27*1023.75/10</f>
+        <v>549.98636443620171</v>
+      </c>
       <c r="K29" s="17"/>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="16"/>
       <c r="B30" s="32" t="s">
-        <v>45</v>
-      </c>
-      <c r="C30" s="17">
-        <f>2*2</f>
-        <v>4</v>
-      </c>
-      <c r="D30" s="33">
-        <f>8/3.281</f>
-        <v>2.4382810118866196</v>
-      </c>
-      <c r="E30" s="17">
-        <v>0.45</v>
-      </c>
-      <c r="F30" s="17">
-        <v>0.9</v>
-      </c>
-      <c r="G30" s="33">
-        <f t="shared" ref="G30:G31" si="3">PRODUCT(C30:F30)</f>
-        <v>3.9500152392563237</v>
-      </c>
+        <v>43</v>
+      </c>
+      <c r="C30" s="17"/>
+      <c r="D30" s="17"/>
+      <c r="E30" s="17"/>
+      <c r="F30" s="17"/>
+      <c r="G30" s="17"/>
       <c r="H30" s="17"/>
       <c r="I30" s="17"/>
-      <c r="J30" s="18"/>
+      <c r="J30" s="18">
+        <f>0.13*G27*348.21/10</f>
+        <v>187.06788958273972</v>
+      </c>
       <c r="K30" s="17"/>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="16"/>
       <c r="B31" s="32" t="s">
-        <v>47</v>
-      </c>
-      <c r="C31" s="17">
-        <f>2*4</f>
-        <v>8</v>
-      </c>
-      <c r="D31" s="33">
-        <v>0.6</v>
-      </c>
-      <c r="E31" s="17">
-        <v>0.6</v>
-      </c>
-      <c r="F31" s="17">
-        <v>0.6</v>
-      </c>
-      <c r="G31" s="33">
-        <f t="shared" si="3"/>
-        <v>1.728</v>
-      </c>
+        <v>44</v>
+      </c>
+      <c r="C31" s="17"/>
+      <c r="D31" s="17"/>
+      <c r="E31" s="17"/>
+      <c r="F31" s="17"/>
+      <c r="G31" s="17"/>
       <c r="H31" s="17"/>
       <c r="I31" s="17"/>
-      <c r="J31" s="18"/>
+      <c r="J31" s="18">
+        <f>0.13*G27*165/10</f>
+        <v>88.642490971402466</v>
+      </c>
       <c r="K31" s="17"/>
     </row>
-    <row r="32" spans="1:11" s="35" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="2"/>
-      <c r="B32" s="40" t="s">
-        <v>36</v>
-      </c>
-      <c r="C32" s="3"/>
-      <c r="D32" s="4"/>
-      <c r="E32" s="5"/>
-      <c r="F32" s="5"/>
-      <c r="G32" s="39">
-        <f>SUM(G30:G31)</f>
-        <v>5.6780152392563235</v>
-      </c>
-      <c r="H32" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="I32" s="6">
-        <v>674.12</v>
-      </c>
-      <c r="J32" s="39">
-        <f>G32*I32</f>
-        <v>3827.6636330874726</v>
-      </c>
-      <c r="K32" s="5"/>
-    </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A33" s="16"/>
-      <c r="B33" s="32"/>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A32" s="16"/>
+      <c r="B32" s="32"/>
+      <c r="C32" s="17"/>
+      <c r="D32" s="17"/>
+      <c r="E32" s="17"/>
+      <c r="F32" s="17"/>
+      <c r="G32" s="17"/>
+      <c r="H32" s="17"/>
+      <c r="I32" s="17"/>
+      <c r="J32" s="18"/>
+      <c r="K32" s="17"/>
+    </row>
+    <row r="33" spans="1:11" ht="30.75" x14ac:dyDescent="0.25">
+      <c r="A33" s="16">
+        <v>3</v>
+      </c>
+      <c r="B33" s="43" t="s">
+        <v>49</v>
+      </c>
       <c r="C33" s="17"/>
       <c r="D33" s="17"/>
       <c r="E33" s="17"/>
@@ -3364,18 +3419,28 @@
       <c r="J33" s="18"/>
       <c r="K33" s="17"/>
     </row>
-    <row r="34" spans="1:11" ht="30.75" x14ac:dyDescent="0.25">
-      <c r="A34" s="16">
-        <v>4</v>
-      </c>
-      <c r="B34" s="43" t="s">
-        <v>50</v>
-      </c>
-      <c r="C34" s="17"/>
-      <c r="D34" s="17"/>
-      <c r="E34" s="17"/>
-      <c r="F34" s="17"/>
-      <c r="G34" s="17"/>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A34" s="16"/>
+      <c r="B34" s="32" t="s">
+        <v>45</v>
+      </c>
+      <c r="C34" s="57">
+        <v>2</v>
+      </c>
+      <c r="D34" s="58">
+        <f>8/3.281</f>
+        <v>2.4382810118866196</v>
+      </c>
+      <c r="E34" s="57">
+        <v>0.45</v>
+      </c>
+      <c r="F34" s="57">
+        <v>0.9</v>
+      </c>
+      <c r="G34" s="58">
+        <f t="shared" ref="G34:G37" si="18">PRODUCT(C34:F34)</f>
+        <v>1.9750076196281618</v>
+      </c>
       <c r="H34" s="17"/>
       <c r="I34" s="17"/>
       <c r="J34" s="18"/>
@@ -3383,28 +3448,23 @@
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" s="16"/>
-      <c r="B35" s="32" t="str">
-        <f>B31</f>
-        <v>-for footing of vertical post</v>
-      </c>
+      <c r="B35" s="32"/>
       <c r="C35" s="17">
-        <f>C31</f>
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="D35" s="33">
-        <f>D31</f>
-        <v>0.6</v>
-      </c>
-      <c r="E35" s="33">
-        <f>E31</f>
-        <v>0.6</v>
-      </c>
-      <c r="F35" s="33">
-        <v>0.15</v>
+        <f>8/3.281</f>
+        <v>2.4382810118866196</v>
+      </c>
+      <c r="E35" s="17">
+        <v>0.45</v>
+      </c>
+      <c r="F35" s="17">
+        <v>0.9</v>
       </c>
       <c r="G35" s="33">
-        <f t="shared" ref="G35:G37" si="4">PRODUCT(C35:F35)</f>
-        <v>0.432</v>
+        <f t="shared" ref="G35" si="19">PRODUCT(C35:F35)</f>
+        <v>0</v>
       </c>
       <c r="H35" s="17"/>
       <c r="I35" s="17"/>
@@ -3414,26 +3474,24 @@
     <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" s="16"/>
       <c r="B36" s="32" t="s">
-        <v>55</v>
-      </c>
-      <c r="C36" s="17">
-        <f>2*1</f>
-        <v>2</v>
-      </c>
-      <c r="D36" s="33">
-        <f>10/3.281</f>
-        <v>3.047851264858275</v>
-      </c>
-      <c r="E36" s="33">
-        <f>12/3.281</f>
-        <v>3.6574215178299299</v>
-      </c>
-      <c r="F36" s="33">
-        <v>0.15</v>
-      </c>
-      <c r="G36" s="33">
-        <f t="shared" si="4"/>
-        <v>3.3441830397713472</v>
+        <v>47</v>
+      </c>
+      <c r="C36" s="57">
+        <f>2*6</f>
+        <v>12</v>
+      </c>
+      <c r="D36" s="58">
+        <v>0.45</v>
+      </c>
+      <c r="E36" s="57">
+        <v>0.45</v>
+      </c>
+      <c r="F36" s="57">
+        <v>0.45</v>
+      </c>
+      <c r="G36" s="58">
+        <f t="shared" si="18"/>
+        <v>1.0935000000000001</v>
       </c>
       <c r="H36" s="17"/>
       <c r="I36" s="17"/>
@@ -3443,26 +3501,25 @@
     <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" s="16"/>
       <c r="B37" s="32" t="s">
-        <v>56</v>
-      </c>
-      <c r="C37" s="17">
-        <f>2*-1</f>
-        <v>-2</v>
-      </c>
-      <c r="D37" s="33">
-        <f>8/3.281</f>
-        <v>2.4382810118866196</v>
-      </c>
-      <c r="E37" s="33">
-        <f>0.6+0.45+0.45</f>
-        <v>1.5</v>
-      </c>
-      <c r="F37" s="33">
-        <v>0.15</v>
-      </c>
-      <c r="G37" s="33">
-        <f t="shared" si="4"/>
-        <v>-1.0972264553489788</v>
+        <v>55</v>
+      </c>
+      <c r="C37" s="57">
+        <v>1</v>
+      </c>
+      <c r="D37" s="58">
+        <f>13/3.281</f>
+        <v>3.9622066443157573</v>
+      </c>
+      <c r="E37" s="58">
+        <f>10/3.281</f>
+        <v>3.047851264858275</v>
+      </c>
+      <c r="F37" s="57">
+        <v>0.1</v>
+      </c>
+      <c r="G37" s="58">
+        <f t="shared" si="18"/>
+        <v>1.2076216532507642</v>
       </c>
       <c r="H37" s="17"/>
       <c r="I37" s="17"/>
@@ -3479,26 +3536,24 @@
       <c r="E38" s="5"/>
       <c r="F38" s="5"/>
       <c r="G38" s="39">
-        <f>SUM(G35:G37)</f>
-        <v>2.6789565844223686</v>
+        <f>SUM(G34:G37)</f>
+        <v>4.2761292728789257</v>
       </c>
       <c r="H38" s="7" t="s">
         <v>46</v>
       </c>
       <c r="I38" s="6">
-        <v>4495.6400000000003</v>
+        <v>674.12</v>
       </c>
       <c r="J38" s="39">
         <f>G38*I38</f>
-        <v>12043.624379192579</v>
+        <v>2882.6242654331413</v>
       </c>
       <c r="K38" s="5"/>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" s="16"/>
-      <c r="B39" s="32" t="s">
-        <v>51</v>
-      </c>
+      <c r="B39" s="32"/>
       <c r="C39" s="17"/>
       <c r="D39" s="17"/>
       <c r="E39" s="17"/>
@@ -3506,16 +3561,15 @@
       <c r="G39" s="17"/>
       <c r="H39" s="17"/>
       <c r="I39" s="17"/>
-      <c r="J39" s="18">
-        <f>0.13*G38*2577.63</f>
-        <v>897.69665189160207</v>
-      </c>
+      <c r="J39" s="18"/>
       <c r="K39" s="17"/>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A40" s="16"/>
-      <c r="B40" s="32" t="s">
-        <v>52</v>
+    <row r="40" spans="1:11" ht="30.75" x14ac:dyDescent="0.25">
+      <c r="A40" s="16">
+        <v>4</v>
+      </c>
+      <c r="B40" s="43" t="s">
+        <v>50</v>
       </c>
       <c r="C40" s="17"/>
       <c r="D40" s="17"/>
@@ -3524,64 +3578,89 @@
       <c r="G40" s="17"/>
       <c r="H40" s="17"/>
       <c r="I40" s="17"/>
-      <c r="J40" s="18">
-        <f>0.13*G38*515.52</f>
-        <v>179.53724079218455</v>
-      </c>
+      <c r="J40" s="18"/>
       <c r="K40" s="17"/>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" s="16"/>
-      <c r="B41" s="42"/>
-      <c r="C41" s="17"/>
-      <c r="D41" s="17"/>
-      <c r="E41" s="17"/>
-      <c r="F41" s="17"/>
-      <c r="G41" s="17"/>
+      <c r="B41" s="32" t="str">
+        <f>B36</f>
+        <v>-for footing of vertical post</v>
+      </c>
+      <c r="C41" s="57">
+        <f>C36</f>
+        <v>12</v>
+      </c>
+      <c r="D41" s="58">
+        <f>D36</f>
+        <v>0.45</v>
+      </c>
+      <c r="E41" s="58">
+        <f>E36</f>
+        <v>0.45</v>
+      </c>
+      <c r="F41" s="58">
+        <v>0.15</v>
+      </c>
+      <c r="G41" s="58">
+        <f t="shared" ref="G41:G44" si="20">PRODUCT(C41:F41)</f>
+        <v>0.36449999999999999</v>
+      </c>
       <c r="H41" s="17"/>
       <c r="I41" s="17"/>
       <c r="J41" s="18"/>
       <c r="K41" s="17"/>
     </row>
-    <row r="42" spans="1:11" ht="30.75" x14ac:dyDescent="0.25">
-      <c r="A42" s="16">
-        <v>5</v>
-      </c>
-      <c r="B42" s="43" t="s">
-        <v>53</v>
-      </c>
-      <c r="C42" s="17"/>
-      <c r="D42" s="17"/>
-      <c r="E42" s="17"/>
-      <c r="F42" s="17"/>
-      <c r="G42" s="17"/>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A42" s="16"/>
+      <c r="B42" s="65" t="s">
+        <v>55</v>
+      </c>
+      <c r="C42" s="57">
+        <f>C52</f>
+        <v>1</v>
+      </c>
+      <c r="D42" s="58">
+        <f>D52</f>
+        <v>3.5</v>
+      </c>
+      <c r="E42" s="58">
+        <f>E52</f>
+        <v>3.9</v>
+      </c>
+      <c r="F42" s="58">
+        <v>0.15</v>
+      </c>
+      <c r="G42" s="58">
+        <f t="shared" si="20"/>
+        <v>2.0474999999999999</v>
+      </c>
       <c r="H42" s="17"/>
       <c r="I42" s="17"/>
-      <c r="J42" s="17"/>
+      <c r="J42" s="18"/>
       <c r="K42" s="17"/>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" s="16"/>
-      <c r="B43" s="32" t="str">
-        <f>B35</f>
-        <v>-for footing of vertical post</v>
-      </c>
-      <c r="C43" s="17">
-        <f>2*4</f>
-        <v>8</v>
-      </c>
-      <c r="D43" s="33">
-        <v>0.6</v>
-      </c>
-      <c r="E43" s="17">
-        <v>0.6</v>
-      </c>
-      <c r="F43" s="33">
-        <v>7.4999999999999997E-2</v>
-      </c>
-      <c r="G43" s="33">
-        <f t="shared" ref="G43:G46" si="5">PRODUCT(C43:F43)</f>
-        <v>0.216</v>
+      <c r="B43" s="65"/>
+      <c r="C43" s="57">
+        <f>C53</f>
+        <v>1</v>
+      </c>
+      <c r="D43" s="58">
+        <f>D53</f>
+        <v>4.2</v>
+      </c>
+      <c r="E43" s="58">
+        <f>E53</f>
+        <v>3.2</v>
+      </c>
+      <c r="F43" s="58">
+        <v>0.15</v>
+      </c>
+      <c r="G43" s="58">
+        <f t="shared" ref="G43" si="21">PRODUCT(C43:F43)</f>
+        <v>2.016</v>
       </c>
       <c r="H43" s="17"/>
       <c r="I43" s="17"/>
@@ -3590,118 +3669,97 @@
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" s="16"/>
-      <c r="B44" s="32"/>
-      <c r="C44" s="17">
-        <f>2*4</f>
-        <v>8</v>
-      </c>
-      <c r="D44" s="33">
-        <v>0.45</v>
-      </c>
-      <c r="E44" s="17">
-        <v>0.45</v>
-      </c>
-      <c r="F44" s="33">
-        <v>0.45</v>
-      </c>
-      <c r="G44" s="33">
-        <f t="shared" si="5"/>
-        <v>0.72900000000000009</v>
+      <c r="B44" s="65" t="s">
+        <v>56</v>
+      </c>
+      <c r="C44" s="57">
+        <f>C54</f>
+        <v>-1</v>
+      </c>
+      <c r="D44" s="58">
+        <f>D54</f>
+        <v>3</v>
+      </c>
+      <c r="E44" s="58">
+        <f>E54</f>
+        <v>1.5</v>
+      </c>
+      <c r="F44" s="58">
+        <v>0.15</v>
+      </c>
+      <c r="G44" s="58">
+        <f t="shared" si="20"/>
+        <v>-0.67499999999999993</v>
       </c>
       <c r="H44" s="17"/>
       <c r="I44" s="17"/>
       <c r="J44" s="18"/>
       <c r="K44" s="17"/>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A45" s="16"/>
-      <c r="B45" s="32" t="str">
-        <f>B36</f>
-        <v>-for flooring</v>
-      </c>
-      <c r="C45" s="17">
-        <f>C36</f>
-        <v>2</v>
-      </c>
-      <c r="D45" s="33">
-        <f>D36</f>
-        <v>3.047851264858275</v>
-      </c>
-      <c r="E45" s="33">
-        <f>E36</f>
-        <v>3.6574215178299299</v>
-      </c>
-      <c r="F45" s="33">
-        <v>0.1</v>
-      </c>
-      <c r="G45" s="33">
-        <f t="shared" si="5"/>
-        <v>2.2294553598475648</v>
-      </c>
-      <c r="H45" s="17"/>
-      <c r="I45" s="17"/>
-      <c r="J45" s="18"/>
-      <c r="K45" s="17"/>
+    <row r="45" spans="1:11" s="35" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="2"/>
+      <c r="B45" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="C45" s="3"/>
+      <c r="D45" s="4"/>
+      <c r="E45" s="5"/>
+      <c r="F45" s="5"/>
+      <c r="G45" s="39">
+        <f>SUM(G41:G44)</f>
+        <v>3.7530000000000001</v>
+      </c>
+      <c r="H45" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="I45" s="6">
+        <v>4495.6400000000003</v>
+      </c>
+      <c r="J45" s="39">
+        <f>G45*I45</f>
+        <v>16872.136920000001</v>
+      </c>
+      <c r="K45" s="5"/>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" s="16"/>
       <c r="B46" s="32" t="s">
-        <v>56</v>
-      </c>
-      <c r="C46" s="17">
-        <f>C37</f>
-        <v>-2</v>
-      </c>
-      <c r="D46" s="33">
-        <f>12/3.281</f>
-        <v>3.6574215178299299</v>
-      </c>
-      <c r="E46" s="33">
-        <f>0.6+0.45+0.45</f>
-        <v>1.5</v>
-      </c>
-      <c r="F46" s="33">
-        <v>0.1</v>
-      </c>
-      <c r="G46" s="33">
-        <f t="shared" si="5"/>
-        <v>-1.097226455348979</v>
-      </c>
+        <v>51</v>
+      </c>
+      <c r="C46" s="17"/>
+      <c r="D46" s="17"/>
+      <c r="E46" s="17"/>
+      <c r="F46" s="17"/>
+      <c r="G46" s="17"/>
       <c r="H46" s="17"/>
       <c r="I46" s="17"/>
-      <c r="J46" s="18"/>
+      <c r="J46" s="18">
+        <f>0.13*G45*2577.63</f>
+        <v>1257.5999007000003</v>
+      </c>
       <c r="K46" s="17"/>
     </row>
-    <row r="47" spans="1:11" s="35" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="2"/>
-      <c r="B47" s="40" t="s">
-        <v>36</v>
-      </c>
-      <c r="C47" s="3"/>
-      <c r="D47" s="4"/>
-      <c r="E47" s="5"/>
-      <c r="F47" s="5"/>
-      <c r="G47" s="39">
-        <f>SUM(G43:G46)</f>
-        <v>2.0772289044985861</v>
-      </c>
-      <c r="H47" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="I47" s="6">
-        <v>13351.1</v>
-      </c>
-      <c r="J47" s="39">
-        <f>G47*I47</f>
-        <v>27733.290826851073</v>
-      </c>
-      <c r="K47" s="5"/>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A47" s="16"/>
+      <c r="B47" s="32" t="s">
+        <v>52</v>
+      </c>
+      <c r="C47" s="17"/>
+      <c r="D47" s="17"/>
+      <c r="E47" s="17"/>
+      <c r="F47" s="17"/>
+      <c r="G47" s="17"/>
+      <c r="H47" s="17"/>
+      <c r="I47" s="17"/>
+      <c r="J47" s="18">
+        <f>0.13*G45*515.52</f>
+        <v>251.51705280000002</v>
+      </c>
+      <c r="K47" s="17"/>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" s="16"/>
-      <c r="B48" s="32" t="s">
-        <v>26</v>
-      </c>
+      <c r="B48" s="42"/>
       <c r="C48" s="17"/>
       <c r="D48" s="17"/>
       <c r="E48" s="17"/>
@@ -3709,16 +3767,15 @@
       <c r="G48" s="17"/>
       <c r="H48" s="17"/>
       <c r="I48" s="17"/>
-      <c r="J48" s="18">
-        <f>0.13*G47*4169.92</f>
-        <v>1126.0441859480768</v>
-      </c>
+      <c r="J48" s="18"/>
       <c r="K48" s="17"/>
     </row>
-    <row r="49" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A49" s="16"/>
-      <c r="B49" s="32" t="s">
-        <v>27</v>
+    <row r="49" spans="1:16" ht="30.75" x14ac:dyDescent="0.25">
+      <c r="A49" s="16">
+        <v>5</v>
+      </c>
+      <c r="B49" s="43" t="s">
+        <v>53</v>
       </c>
       <c r="C49" s="17"/>
       <c r="D49" s="17"/>
@@ -3727,148 +3784,168 @@
       <c r="G49" s="17"/>
       <c r="H49" s="17"/>
       <c r="I49" s="17"/>
-      <c r="J49" s="18">
-        <f>0.13*G47*1414.16</f>
-        <v>381.87942358614367</v>
-      </c>
+      <c r="J49" s="17"/>
       <c r="K49" s="17"/>
     </row>
-    <row r="50" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A50" s="16"/>
-      <c r="B50" s="32" t="s">
-        <v>28</v>
-      </c>
-      <c r="C50" s="17"/>
-      <c r="D50" s="17"/>
-      <c r="E50" s="17"/>
-      <c r="F50" s="17"/>
-      <c r="G50" s="17"/>
+      <c r="B50" s="32" t="str">
+        <f>B41</f>
+        <v>-for footing of vertical post</v>
+      </c>
+      <c r="C50" s="57">
+        <f>C36</f>
+        <v>12</v>
+      </c>
+      <c r="D50" s="58">
+        <v>0.45</v>
+      </c>
+      <c r="E50" s="57">
+        <v>0.45</v>
+      </c>
+      <c r="F50" s="58">
+        <v>7.4999999999999997E-2</v>
+      </c>
+      <c r="G50" s="58">
+        <f t="shared" ref="G50:G54" si="22">PRODUCT(C50:F50)</f>
+        <v>0.18225</v>
+      </c>
       <c r="H50" s="17"/>
       <c r="I50" s="17"/>
-      <c r="J50" s="18">
-        <f>0.13*G47*(1652.5+737.97+349.56)</f>
-        <v>739.91703697512401</v>
-      </c>
+      <c r="J50" s="18"/>
       <c r="K50" s="17"/>
     </row>
-    <row r="51" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A51" s="16"/>
-      <c r="B51" s="32" t="s">
-        <v>30</v>
-      </c>
-      <c r="C51" s="17"/>
-      <c r="D51" s="17"/>
-      <c r="E51" s="17"/>
-      <c r="F51" s="17"/>
-      <c r="G51" s="17"/>
+      <c r="B51" s="32"/>
+      <c r="C51" s="17">
+        <v>0</v>
+      </c>
+      <c r="D51" s="33">
+        <v>0.45</v>
+      </c>
+      <c r="E51" s="17">
+        <v>0.45</v>
+      </c>
+      <c r="F51" s="33">
+        <v>0.45</v>
+      </c>
+      <c r="G51" s="33">
+        <f t="shared" si="22"/>
+        <v>0</v>
+      </c>
       <c r="H51" s="17"/>
       <c r="I51" s="17"/>
-      <c r="J51" s="18">
-        <f>0.13*G47*42</f>
-        <v>11.341669818562281</v>
-      </c>
+      <c r="J51" s="18"/>
       <c r="K51" s="17"/>
     </row>
-    <row r="52" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A52" s="16"/>
-      <c r="B52" s="32"/>
-      <c r="C52" s="17"/>
-      <c r="D52" s="17"/>
-      <c r="E52" s="17"/>
-      <c r="F52" s="17"/>
-      <c r="G52" s="17"/>
+      <c r="B52" s="32" t="str">
+        <f>B42</f>
+        <v>-for flooring</v>
+      </c>
+      <c r="C52" s="57">
+        <v>1</v>
+      </c>
+      <c r="D52" s="58">
+        <v>3.5</v>
+      </c>
+      <c r="E52" s="58">
+        <v>3.9</v>
+      </c>
+      <c r="F52" s="58">
+        <v>7.4999999999999997E-2</v>
+      </c>
+      <c r="G52" s="58">
+        <f t="shared" si="22"/>
+        <v>1.0237499999999999</v>
+      </c>
       <c r="H52" s="17"/>
       <c r="I52" s="17"/>
       <c r="J52" s="18"/>
       <c r="K52" s="17"/>
     </row>
-    <row r="53" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A53" s="16">
-        <v>6</v>
-      </c>
-      <c r="B53" s="43" t="s">
-        <v>54</v>
-      </c>
-      <c r="C53" s="17"/>
-      <c r="D53" s="17"/>
-      <c r="E53" s="17"/>
-      <c r="F53" s="17"/>
-      <c r="G53" s="17"/>
+    <row r="53" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A53" s="16"/>
+      <c r="B53" s="32"/>
+      <c r="C53" s="57">
+        <v>1</v>
+      </c>
+      <c r="D53" s="58">
+        <v>4.2</v>
+      </c>
+      <c r="E53" s="58">
+        <v>3.2</v>
+      </c>
+      <c r="F53" s="58">
+        <v>0.1</v>
+      </c>
+      <c r="G53" s="58">
+        <f t="shared" si="22"/>
+        <v>1.3440000000000003</v>
+      </c>
       <c r="H53" s="17"/>
       <c r="I53" s="17"/>
-      <c r="J53" s="17"/>
+      <c r="J53" s="18"/>
       <c r="K53" s="17"/>
     </row>
-    <row r="54" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A54" s="16"/>
       <c r="B54" s="32" t="s">
-        <v>45</v>
-      </c>
-      <c r="C54" s="17">
-        <f>2*2</f>
-        <v>4</v>
-      </c>
-      <c r="D54" s="33">
-        <f>8/3.281</f>
-        <v>2.4382810118866196</v>
-      </c>
-      <c r="E54" s="33">
-        <v>0.45</v>
-      </c>
-      <c r="F54" s="33">
-        <v>0.9</v>
-      </c>
-      <c r="G54" s="33">
-        <f>PRODUCT(C54:F54)</f>
-        <v>3.9500152392563237</v>
+        <v>56</v>
+      </c>
+      <c r="C54" s="57">
+        <v>-1</v>
+      </c>
+      <c r="D54" s="58">
+        <v>3</v>
+      </c>
+      <c r="E54" s="58">
+        <f>0.6+0.45+0.45</f>
+        <v>1.5</v>
+      </c>
+      <c r="F54" s="58">
+        <v>0.1</v>
+      </c>
+      <c r="G54" s="58">
+        <f t="shared" si="22"/>
+        <v>-0.45</v>
       </c>
       <c r="H54" s="17"/>
       <c r="I54" s="17"/>
-      <c r="J54" s="17"/>
+      <c r="J54" s="18"/>
       <c r="K54" s="17"/>
-      <c r="M54" s="33">
-        <f>7</f>
-        <v>7</v>
-      </c>
-      <c r="N54" s="33">
-        <f>2</f>
-        <v>2</v>
-      </c>
-      <c r="O54" s="33"/>
-      <c r="P54" s="33">
-        <f>PI()*M54*SQRT(M54^2+N54^2)</f>
-        <v>160.09797821843054</v>
-      </c>
-    </row>
-    <row r="55" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="55" spans="1:16" s="35" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" s="2"/>
-      <c r="B55" s="34" t="s">
-        <v>16</v>
+      <c r="B55" s="40" t="s">
+        <v>36</v>
       </c>
       <c r="C55" s="3"/>
       <c r="D55" s="4"/>
       <c r="E55" s="5"/>
       <c r="F55" s="5"/>
-      <c r="G55" s="6">
-        <f>SUM(G54:G54)</f>
-        <v>3.9500152392563237</v>
+      <c r="G55" s="39">
+        <f>SUM(G50:G54)</f>
+        <v>2.1</v>
       </c>
       <c r="H55" s="7" t="s">
         <v>46</v>
       </c>
       <c r="I55" s="6">
-        <v>6337.3</v>
-      </c>
-      <c r="J55" s="18">
+        <v>13351.1</v>
+      </c>
+      <c r="J55" s="39">
         <f>G55*I55</f>
-        <v>25032.431575739101</v>
+        <v>28037.31</v>
       </c>
       <c r="K55" s="5"/>
     </row>
-    <row r="56" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A56" s="16"/>
       <c r="B56" s="32" t="s">
-        <v>51</v>
+        <v>26</v>
       </c>
       <c r="C56" s="17"/>
       <c r="D56" s="17"/>
@@ -3878,15 +3955,15 @@
       <c r="H56" s="17"/>
       <c r="I56" s="17"/>
       <c r="J56" s="18">
-        <f>0.13*G55*2577.63</f>
-        <v>1323.6181115513564</v>
+        <f>0.13*G55*4169.92</f>
+        <v>1138.3881600000002</v>
       </c>
       <c r="K56" s="17"/>
     </row>
-    <row r="57" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A57" s="16"/>
       <c r="B57" s="32" t="s">
-        <v>52</v>
+        <v>27</v>
       </c>
       <c r="C57" s="17"/>
       <c r="D57" s="17"/>
@@ -3896,15 +3973,15 @@
       <c r="H57" s="17"/>
       <c r="I57" s="17"/>
       <c r="J57" s="18">
-        <f>0.13*G55*257.76</f>
-        <v>132.3602706491923</v>
+        <f>0.13*G55*1414.16</f>
+        <v>386.06568000000004</v>
       </c>
       <c r="K57" s="17"/>
     </row>
-    <row r="58" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A58" s="16"/>
       <c r="B58" s="32" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C58" s="17"/>
       <c r="D58" s="17"/>
@@ -3914,12 +3991,12 @@
       <c r="H58" s="17"/>
       <c r="I58" s="17"/>
       <c r="J58" s="18">
-        <f>0.13*G55*133.56</f>
-        <v>68.583324596159699</v>
+        <f>0.13*G55*(1652.5+737.97+349.56)</f>
+        <v>748.02819000000011</v>
       </c>
       <c r="K58" s="17"/>
     </row>
-    <row r="59" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A59" s="16"/>
       <c r="B59" s="32" t="s">
         <v>30</v>
@@ -3932,12 +4009,12 @@
       <c r="H59" s="17"/>
       <c r="I59" s="17"/>
       <c r="J59" s="18">
-        <f>0.13*G55*19.6</f>
-        <v>10.064638829625114</v>
+        <f>0.13*G55*42</f>
+        <v>11.466000000000001</v>
       </c>
       <c r="K59" s="17"/>
     </row>
-    <row r="60" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A60" s="16"/>
       <c r="B60" s="32"/>
       <c r="C60" s="17"/>
@@ -3950,183 +4027,377 @@
       <c r="J60" s="18"/>
       <c r="K60" s="17"/>
     </row>
-    <row r="61" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="2">
+    <row r="61" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A61" s="16">
+        <v>6</v>
+      </c>
+      <c r="B61" s="43" t="s">
+        <v>54</v>
+      </c>
+      <c r="C61" s="17"/>
+      <c r="D61" s="17"/>
+      <c r="E61" s="17"/>
+      <c r="F61" s="17"/>
+      <c r="G61" s="17"/>
+      <c r="H61" s="17"/>
+      <c r="I61" s="17"/>
+      <c r="J61" s="17"/>
+      <c r="K61" s="17"/>
+    </row>
+    <row r="62" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A62" s="16"/>
+      <c r="B62" s="32" t="s">
+        <v>45</v>
+      </c>
+      <c r="C62" s="57">
+        <v>2</v>
+      </c>
+      <c r="D62" s="58">
+        <v>3</v>
+      </c>
+      <c r="E62" s="58">
+        <v>0.45</v>
+      </c>
+      <c r="F62" s="58">
+        <v>0.9</v>
+      </c>
+      <c r="G62" s="58">
+        <f>PRODUCT(C62:F62)</f>
+        <v>2.4300000000000002</v>
+      </c>
+      <c r="H62" s="17"/>
+      <c r="I62" s="17"/>
+      <c r="J62" s="17"/>
+      <c r="K62" s="17"/>
+      <c r="M62" s="33">
+        <f>7</f>
         <v>7</v>
       </c>
-      <c r="B61" s="1" t="s">
+      <c r="N62" s="33">
+        <f>2</f>
+        <v>2</v>
+      </c>
+      <c r="O62" s="33"/>
+      <c r="P62" s="33">
+        <f>PI()*M62*SQRT(M62^2+N62^2)</f>
+        <v>160.09797821843054</v>
+      </c>
+    </row>
+    <row r="63" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A63" s="16"/>
+      <c r="B63" s="32"/>
+      <c r="C63" s="17">
+        <v>0</v>
+      </c>
+      <c r="D63" s="33">
+        <v>3</v>
+      </c>
+      <c r="E63" s="33">
+        <v>0.45</v>
+      </c>
+      <c r="F63" s="33">
+        <v>0.9</v>
+      </c>
+      <c r="G63" s="33">
+        <f>PRODUCT(C63:F63)</f>
+        <v>0</v>
+      </c>
+      <c r="H63" s="17"/>
+      <c r="I63" s="17"/>
+      <c r="J63" s="17"/>
+      <c r="K63" s="17"/>
+      <c r="M63" s="59"/>
+      <c r="N63" s="59"/>
+      <c r="O63" s="59"/>
+      <c r="P63" s="59"/>
+    </row>
+    <row r="64" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A64" s="2"/>
+      <c r="B64" s="34" t="s">
+        <v>16</v>
+      </c>
+      <c r="C64" s="3"/>
+      <c r="D64" s="4"/>
+      <c r="E64" s="5"/>
+      <c r="F64" s="5"/>
+      <c r="G64" s="6">
+        <f>SUM(G62:G62)</f>
+        <v>2.4300000000000002</v>
+      </c>
+      <c r="H64" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="I64" s="6">
+        <v>6337.3</v>
+      </c>
+      <c r="J64" s="18">
+        <f>G64*I64</f>
+        <v>15399.639000000001</v>
+      </c>
+      <c r="K64" s="5"/>
+    </row>
+    <row r="65" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A65" s="16"/>
+      <c r="B65" s="32" t="s">
+        <v>51</v>
+      </c>
+      <c r="C65" s="17"/>
+      <c r="D65" s="17"/>
+      <c r="E65" s="17"/>
+      <c r="F65" s="17"/>
+      <c r="G65" s="17"/>
+      <c r="H65" s="17"/>
+      <c r="I65" s="17"/>
+      <c r="J65" s="18">
+        <f>0.13*G64*2577.63</f>
+        <v>814.27331700000002</v>
+      </c>
+      <c r="K65" s="17"/>
+    </row>
+    <row r="66" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A66" s="16"/>
+      <c r="B66" s="32" t="s">
+        <v>52</v>
+      </c>
+      <c r="C66" s="17"/>
+      <c r="D66" s="17"/>
+      <c r="E66" s="17"/>
+      <c r="F66" s="17"/>
+      <c r="G66" s="17"/>
+      <c r="H66" s="17"/>
+      <c r="I66" s="17"/>
+      <c r="J66" s="18">
+        <f>0.13*G64*257.76</f>
+        <v>81.426383999999999</v>
+      </c>
+      <c r="K66" s="17"/>
+    </row>
+    <row r="67" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A67" s="16"/>
+      <c r="B67" s="32" t="s">
+        <v>29</v>
+      </c>
+      <c r="C67" s="17"/>
+      <c r="D67" s="17"/>
+      <c r="E67" s="17"/>
+      <c r="F67" s="17"/>
+      <c r="G67" s="17"/>
+      <c r="H67" s="17"/>
+      <c r="I67" s="17"/>
+      <c r="J67" s="18">
+        <f>0.13*G64*133.56</f>
+        <v>42.191604000000005</v>
+      </c>
+      <c r="K67" s="17"/>
+    </row>
+    <row r="68" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A68" s="16"/>
+      <c r="B68" s="32" t="s">
+        <v>30</v>
+      </c>
+      <c r="C68" s="17"/>
+      <c r="D68" s="17"/>
+      <c r="E68" s="17"/>
+      <c r="F68" s="17"/>
+      <c r="G68" s="17"/>
+      <c r="H68" s="17"/>
+      <c r="I68" s="17"/>
+      <c r="J68" s="18">
+        <f>0.13*G64*19.6</f>
+        <v>6.1916400000000005</v>
+      </c>
+      <c r="K68" s="17"/>
+    </row>
+    <row r="69" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A69" s="16"/>
+      <c r="B69" s="32"/>
+      <c r="C69" s="17"/>
+      <c r="D69" s="17"/>
+      <c r="E69" s="17"/>
+      <c r="F69" s="17"/>
+      <c r="G69" s="17"/>
+      <c r="H69" s="17"/>
+      <c r="I69" s="17"/>
+      <c r="J69" s="18"/>
+      <c r="K69" s="17"/>
+    </row>
+    <row r="70" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A70" s="2">
+        <v>7</v>
+      </c>
+      <c r="B70" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C61" s="3">
+      <c r="C70" s="3">
         <v>1</v>
       </c>
-      <c r="D61" s="4"/>
-      <c r="E61" s="5"/>
-      <c r="F61" s="5"/>
-      <c r="G61" s="7">
-        <f t="shared" ref="G61" si="6">PRODUCT(C61:F61)</f>
+      <c r="D70" s="4"/>
+      <c r="E70" s="5"/>
+      <c r="F70" s="5"/>
+      <c r="G70" s="7">
+        <f t="shared" ref="G70" si="23">PRODUCT(C70:F70)</f>
         <v>1</v>
       </c>
-      <c r="H61" s="7" t="s">
+      <c r="H70" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="I61" s="6">
+      <c r="I70" s="6">
         <v>1000</v>
       </c>
-      <c r="J61" s="7">
-        <f>G61*I61</f>
+      <c r="J70" s="7">
+        <f>G70*I70</f>
         <v>1000</v>
       </c>
-      <c r="K61" s="5"/>
-    </row>
-    <row r="62" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A62" s="2"/>
-      <c r="B62" s="8"/>
-      <c r="C62" s="3"/>
-      <c r="D62" s="4"/>
-      <c r="E62" s="5"/>
-      <c r="F62" s="5"/>
-      <c r="G62" s="6"/>
-      <c r="H62" s="7"/>
-      <c r="I62" s="6"/>
-      <c r="J62" s="18"/>
-      <c r="K62" s="5"/>
-    </row>
-    <row r="63" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A63" s="21"/>
-      <c r="B63" s="22" t="s">
+      <c r="K70" s="5"/>
+    </row>
+    <row r="71" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A71" s="2"/>
+      <c r="B71" s="8"/>
+      <c r="C71" s="3"/>
+      <c r="D71" s="4"/>
+      <c r="E71" s="5"/>
+      <c r="F71" s="5"/>
+      <c r="G71" s="6"/>
+      <c r="H71" s="7"/>
+      <c r="I71" s="6"/>
+      <c r="J71" s="18"/>
+      <c r="K71" s="5"/>
+    </row>
+    <row r="72" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A72" s="21"/>
+      <c r="B72" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="C63" s="23"/>
-      <c r="D63" s="24"/>
-      <c r="E63" s="24"/>
-      <c r="F63" s="24"/>
-      <c r="G63" s="18"/>
-      <c r="H63" s="18"/>
-      <c r="I63" s="18"/>
-      <c r="J63" s="18">
-        <f>SUM(J9:J61)</f>
-        <v>234835.07491669987</v>
-      </c>
-      <c r="K63" s="25"/>
-    </row>
-    <row r="64" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="M64" s="20"/>
-      <c r="N64" s="20"/>
-      <c r="O64" s="20"/>
-      <c r="P64" s="20"/>
-      <c r="Q64" s="20"/>
-      <c r="R64" s="20"/>
-      <c r="S64" s="20"/>
-    </row>
-    <row r="65" spans="1:19" s="20" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="26"/>
-      <c r="B65" s="27" t="s">
+      <c r="C72" s="23"/>
+      <c r="D72" s="24"/>
+      <c r="E72" s="24"/>
+      <c r="F72" s="24"/>
+      <c r="G72" s="18"/>
+      <c r="H72" s="18"/>
+      <c r="I72" s="18"/>
+      <c r="J72" s="18">
+        <f>SUM(J9:J70)</f>
+        <v>171041.49224446158</v>
+      </c>
+      <c r="K72" s="25"/>
+    </row>
+    <row r="73" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="M73" s="20"/>
+      <c r="N73" s="20"/>
+      <c r="O73" s="20"/>
+      <c r="P73" s="20"/>
+      <c r="Q73" s="20"/>
+      <c r="R73" s="20"/>
+      <c r="S73" s="20"/>
+    </row>
+    <row r="74" spans="1:19" s="20" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A74" s="26"/>
+      <c r="B74" s="27" t="s">
         <v>64</v>
       </c>
-      <c r="C65" s="50">
-        <f>J63</f>
-        <v>234835.07491669987</v>
-      </c>
-      <c r="D65" s="51"/>
-      <c r="E65" s="9">
+      <c r="C74" s="44">
+        <f>J72</f>
+        <v>171041.49224446158</v>
+      </c>
+      <c r="D74" s="45"/>
+      <c r="E74" s="9">
         <v>100</v>
       </c>
-      <c r="F65" s="26"/>
-      <c r="G65" s="28"/>
-      <c r="H65" s="26"/>
-      <c r="I65" s="29"/>
-      <c r="J65" s="30"/>
-      <c r="K65" s="31"/>
-      <c r="M65" s="19"/>
-      <c r="N65" s="19"/>
-      <c r="O65" s="19"/>
-      <c r="P65" s="19"/>
-      <c r="Q65" s="19"/>
-      <c r="R65" s="19"/>
-      <c r="S65" s="19"/>
-    </row>
-    <row r="66" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B66" s="27" t="s">
+      <c r="F74" s="26"/>
+      <c r="G74" s="28"/>
+      <c r="H74" s="26"/>
+      <c r="I74" s="29"/>
+      <c r="J74" s="30"/>
+      <c r="K74" s="31"/>
+      <c r="M74" s="19"/>
+      <c r="N74" s="19"/>
+      <c r="O74" s="19"/>
+      <c r="P74" s="19"/>
+      <c r="Q74" s="19"/>
+      <c r="R74" s="19"/>
+      <c r="S74" s="19"/>
+    </row>
+    <row r="75" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B75" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="C66" s="54">
+      <c r="C75" s="48">
         <v>200000</v>
       </c>
-      <c r="D66" s="55"/>
-      <c r="E66" s="9"/>
-    </row>
-    <row r="67" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B67" s="27" t="s">
+      <c r="D75" s="49"/>
+      <c r="E75" s="9"/>
+    </row>
+    <row r="76" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B76" s="27" t="s">
         <v>22</v>
       </c>
-      <c r="C67" s="54">
-        <f>C66-C69-C70</f>
+      <c r="C76" s="48">
+        <f>C75-C78-C79</f>
         <v>190000</v>
       </c>
-      <c r="D67" s="55"/>
-      <c r="E67" s="9">
-        <f>C67/C65*100</f>
-        <v>80.907845673137345</v>
-      </c>
-    </row>
-    <row r="68" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B68" s="27" t="s">
+      <c r="D76" s="49"/>
+      <c r="E76" s="9">
+        <f>C76/C74*100</f>
+        <v>111.08415712863516</v>
+      </c>
+    </row>
+    <row r="77" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B77" s="27" t="s">
         <v>31</v>
       </c>
-      <c r="C68" s="56">
-        <f>C65-C67</f>
-        <v>44835.074916699872</v>
-      </c>
-      <c r="D68" s="56"/>
-      <c r="E68" s="9">
-        <f>100-E67</f>
-        <v>19.092154326862655</v>
-      </c>
-    </row>
-    <row r="69" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B69" s="27" t="s">
+      <c r="C77" s="50">
+        <f>C74-C76</f>
+        <v>-18958.50775553842</v>
+      </c>
+      <c r="D77" s="50"/>
+      <c r="E77" s="9">
+        <f>100-E76</f>
+        <v>-11.084157128635155</v>
+      </c>
+    </row>
+    <row r="78" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B78" s="27" t="s">
         <v>23</v>
       </c>
-      <c r="C69" s="50">
-        <f>C66*0.03</f>
+      <c r="C78" s="44">
+        <f>C75*0.03</f>
         <v>6000</v>
       </c>
-      <c r="D69" s="51"/>
-      <c r="E69" s="9">
+      <c r="D78" s="45"/>
+      <c r="E78" s="9">
         <v>3</v>
       </c>
     </row>
-    <row r="70" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B70" s="27" t="s">
+    <row r="79" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B79" s="27" t="s">
         <v>24</v>
       </c>
-      <c r="C70" s="50">
-        <f>C66*0.02</f>
+      <c r="C79" s="44">
+        <f>C75*0.02</f>
         <v>4000</v>
       </c>
-      <c r="D70" s="51"/>
-      <c r="E70" s="9">
+      <c r="D79" s="45"/>
+      <c r="E79" s="9">
         <v>2</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="C69:D69"/>
-    <mergeCell ref="C70:D70"/>
-    <mergeCell ref="A7:F7"/>
-    <mergeCell ref="H7:K7"/>
-    <mergeCell ref="C65:D65"/>
-    <mergeCell ref="C66:D66"/>
-    <mergeCell ref="C67:D67"/>
-    <mergeCell ref="C68:D68"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="H6:K6"/>
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="A3:K3"/>
     <mergeCell ref="A4:K4"/>
     <mergeCell ref="A5:K5"/>
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="H6:K6"/>
+    <mergeCell ref="C78:D78"/>
+    <mergeCell ref="C79:D79"/>
+    <mergeCell ref="A7:F7"/>
+    <mergeCell ref="H7:K7"/>
+    <mergeCell ref="C74:D74"/>
+    <mergeCell ref="C75:D75"/>
+    <mergeCell ref="C76:D76"/>
+    <mergeCell ref="C77:D77"/>
   </mergeCells>
   <pageMargins left="0.70866141732283505" right="0.70866141732283505" top="0.74803149606299202" bottom="0.74803149606299202" header="0.31496062992126" footer="0.31496062992126"/>
   <pageSetup paperSize="9" scale="80" orientation="portrait" verticalDpi="1200" r:id="rId1"/>
@@ -4134,7 +4405,7 @@
     <oddFooter>&amp;LPrepared By:&amp;CChecked By:&amp;RApproved By:</oddFooter>
   </headerFooter>
   <rowBreaks count="1" manualBreakCount="1">
-    <brk id="45" max="10" man="1"/>
+    <brk id="53" max="10" man="1"/>
   </rowBreaks>
 </worksheet>
 </file>
</xml_diff>